<commit_message>
fix(docs): xlsx opens clean in Excel (no 'Repaired' prompt)
Add docProps/core.xml and docProps/app.xml (+ Content_Types overrides and
root relationships) and complete the workbook (bookViews, calcPr) so Excel
no longer flags the file for repair. Instrucciones sheet already reflects the
flat titled-table layout.
</commit_message>
<xml_diff>
--- a/docs/plantilla-productos.xlsx
+++ b/docs/plantilla-productos.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <bookViews>
+    <workbookView activeTab="1"/>
+  </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
     <sheet name="Productos" sheetId="2" r:id="rId2"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 

</xml_diff>